<commit_message>
Atlas: Section naming, one-page section PDFs, uniform label zoom, section labels, decisions digest
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wfTBB8erJev2gayfgdzYG
</commit_message>
<xml_diff>
--- a/h-number-map/site/pdf/Cedar_Grove_H-Map_lots.xlsx
+++ b/h-number-map/site/pdf/Cedar_Grove_H-Map_lots.xlsx
@@ -505,7 +505,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Legacy section and lot are cross-reference only. Burial records are not part of this workbook.</t>
+          <t>Section and lot are the cemetery section letters and lot labels. Burial records are not part of this workbook.</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -538,12 +538,12 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Legacy section</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Legacy lot</t>
+          <t>Lot</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -84355,7 +84355,7 @@
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -84376,12 +84376,12 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Legacy section</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Legacy lot</t>
+          <t>Lot</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -84408,7 +84408,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -84434,7 +84434,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -84460,7 +84460,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -84486,7 +84486,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -84512,7 +84512,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -84538,7 +84538,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -84564,7 +84564,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -84590,7 +84590,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -84616,7 +84616,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -84642,7 +84642,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -84668,7 +84668,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -84694,7 +84694,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -84720,7 +84720,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -84772,7 +84772,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -84798,7 +84798,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -84824,7 +84824,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -84850,7 +84850,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -84876,7 +84876,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -84902,7 +84902,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -84954,7 +84954,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -84980,7 +84980,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -85006,7 +85006,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -85032,7 +85032,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -85058,7 +85058,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -85084,7 +85084,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -85110,7 +85110,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -85136,7 +85136,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -85162,7 +85162,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -85214,7 +85214,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -85240,7 +85240,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -85266,7 +85266,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -85292,7 +85292,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -85318,7 +85318,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -85408,7 +85408,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -85522,7 +85522,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -85548,7 +85548,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -85574,7 +85574,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -85600,7 +85600,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -85626,7 +85626,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -85804,7 +85804,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -85830,7 +85830,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -85856,7 +85856,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -85882,7 +85882,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -85908,7 +85908,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -85934,7 +85934,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -85960,7 +85960,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -86112,7 +86112,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -86150,7 +86150,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -86176,7 +86176,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -86202,7 +86202,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -86228,7 +86228,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -86254,7 +86254,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -86280,7 +86280,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -86318,7 +86318,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -86356,7 +86356,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -86610,7 +86610,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
@@ -86662,7 +86662,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -86700,7 +86700,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -86738,7 +86738,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -86828,7 +86828,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
@@ -86854,7 +86854,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
@@ -86880,7 +86880,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
@@ -86906,7 +86906,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -87010,7 +87010,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -87036,7 +87036,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -87100,7 +87100,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -87138,7 +87138,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -87176,7 +87176,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -87214,7 +87214,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -87252,7 +87252,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -87290,7 +87290,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -87404,7 +87404,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
@@ -87430,7 +87430,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
@@ -87534,7 +87534,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -87598,7 +87598,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -87624,7 +87624,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -87650,7 +87650,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -87702,7 +87702,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -87740,7 +87740,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -87778,7 +87778,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -88740,7 +88740,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -88908,7 +88908,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -89128,7 +89128,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B166" t="inlineStr"/>
@@ -89154,7 +89154,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B167" t="inlineStr"/>
@@ -89180,7 +89180,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B168" t="inlineStr"/>
@@ -89206,7 +89206,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B169" t="inlineStr"/>
@@ -89232,7 +89232,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B170" t="inlineStr"/>
@@ -89452,7 +89452,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -89490,7 +89490,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B179" t="inlineStr"/>
@@ -89880,7 +89880,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B194" t="inlineStr"/>
@@ -89906,7 +89906,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -89944,7 +89944,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -89982,7 +89982,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -90020,7 +90020,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B198" t="inlineStr"/>
@@ -90046,7 +90046,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B199" t="inlineStr"/>
@@ -90072,7 +90072,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B200" t="inlineStr"/>
@@ -90098,7 +90098,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B201" t="inlineStr"/>
@@ -90124,7 +90124,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B202" t="inlineStr"/>
@@ -90150,7 +90150,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -90188,7 +90188,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -90226,7 +90226,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -90264,7 +90264,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Two places on the drawing carry the same legacy label for the same section.</t>
+          <t>Two places on the drawing carry the same lot label for the same section.</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -90302,7 +90302,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B207" t="inlineStr"/>
@@ -90366,7 +90366,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B209" t="inlineStr"/>
@@ -90392,7 +90392,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>The label does not exist in the legacy section this part of the map belongs to.</t>
+          <t>The label does not exist in the section this part of the map belongs to.</t>
         </is>
       </c>
       <c r="B210" t="inlineStr"/>
@@ -90629,7 +90629,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
@@ -90642,12 +90642,12 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Legacy section</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Legacy lot</t>
+          <t>Lot</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">

</xml_diff>